<commit_message>
Review workbook frictionlessness and repair evidence-backed reference defects
</commit_message>
<xml_diff>
--- a/01-meridian-health-grc-program/artifacts/nist_csf_gap_assessment.xlsx
+++ b/01-meridian-health-grc-program/artifacts/nist_csf_gap_assessment.xlsx
@@ -729,12 +729,13 @@
         <f>IF(G5="","",IF(G5&gt;=2,"High",IF(G5=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I5" s="31" t="inlineStr">
+      <c r="I5" s="31" t="n"/>
+      <c r="J5" s="31" t="inlineStr">
         <is>
           <t>Add regulatory-driver field to risk register intake so every risk traces to a specific obligation</t>
         </is>
       </c>
-      <c r="J5" s="31" t="inlineStr">
+      <c r="K5" s="31" t="inlineStr">
         <is>
           <t>Compliance Officer</t>
         </is>
@@ -775,12 +776,13 @@
         <f>IF(G6="","",IF(G6&gt;=2,"High",IF(G6=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I6" s="31" t="inlineStr">
+      <c r="I6" s="31" t="n"/>
+      <c r="J6" s="31" t="inlineStr">
         <is>
           <t>Draft and board-approve a formal risk appetite statement with quantitative thresholds by risk category</t>
         </is>
       </c>
-      <c r="J6" s="31" t="inlineStr">
+      <c r="K6" s="31" t="inlineStr">
         <is>
           <t>CISO</t>
         </is>
@@ -868,12 +870,13 @@
         <f>IF(G8="","",IF(G8&gt;=2,"High",IF(G8=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I8" s="31" t="inlineStr">
+      <c r="I8" s="31" t="n"/>
+      <c r="J8" s="31" t="inlineStr">
         <is>
           <t>Implement policy management tool with automated review reminders and version history</t>
         </is>
       </c>
-      <c r="J8" s="31" t="inlineStr">
+      <c r="K8" s="31" t="inlineStr">
         <is>
           <t>Compliance Officer</t>
         </is>
@@ -914,12 +917,13 @@
         <f>IF(G9="","",IF(G9&gt;=2,"High",IF(G9=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I9" s="31" t="inlineStr">
+      <c r="I9" s="31" t="n"/>
+      <c r="J9" s="31" t="inlineStr">
         <is>
           <t>Institute quarterly board-level cybersecurity risk briefing with standardized reporting template</t>
         </is>
       </c>
-      <c r="J9" s="31" t="inlineStr">
+      <c r="K9" s="31" t="inlineStr">
         <is>
           <t>CISO</t>
         </is>
@@ -960,12 +964,13 @@
         <f>IF(G10="","",IF(G10&gt;=2,"High",IF(G10=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I10" s="31" t="inlineStr">
+      <c r="I10" s="31" t="n"/>
+      <c r="J10" s="31" t="inlineStr">
         <is>
           <t>Deploy TPRM platform; require SOC 2/questionnaire before any vendor onboarding</t>
         </is>
       </c>
-      <c r="J10" s="31" t="inlineStr">
+      <c r="K10" s="31" t="inlineStr">
         <is>
           <t>Vendor Risk Manager</t>
         </is>
@@ -1006,12 +1011,13 @@
         <f>IF(G11="","",IF(G11&gt;=2,"High",IF(G11=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I11" s="31" t="inlineStr">
+      <c r="I11" s="31" t="n"/>
+      <c r="J11" s="31" t="inlineStr">
         <is>
           <t>Deploy SaaS discovery/CASB tooling to close asset visibility gap</t>
         </is>
       </c>
-      <c r="J11" s="31" t="inlineStr">
+      <c r="K11" s="31" t="inlineStr">
         <is>
           <t>IT Asset Manager</t>
         </is>
@@ -1052,12 +1058,13 @@
         <f>IF(G12="","",IF(G12&gt;=2,"High",IF(G12=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I12" s="31" t="inlineStr">
+      <c r="I12" s="31" t="n"/>
+      <c r="J12" s="31" t="inlineStr">
         <is>
           <t>Extend risk assessment to include threat-intelligence-informed likelihood scoring</t>
         </is>
       </c>
-      <c r="J12" s="31" t="inlineStr">
+      <c r="K12" s="31" t="inlineStr">
         <is>
           <t>GRC Analyst</t>
         </is>
@@ -1098,12 +1105,13 @@
         <f>IF(G13="","",IF(G13&gt;=2,"High",IF(G13=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I13" s="31" t="inlineStr">
+      <c r="I13" s="31" t="n"/>
+      <c r="J13" s="31" t="inlineStr">
         <is>
           <t>Stand up CAPA tracker linking incident/audit findings to remediation with due dates and closure verification</t>
         </is>
       </c>
-      <c r="J13" s="31" t="inlineStr">
+      <c r="K13" s="31" t="inlineStr">
         <is>
           <t>CISO</t>
         </is>
@@ -1144,12 +1152,13 @@
         <f>IF(G14="","",IF(G14&gt;=2,"High",IF(G14=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I14" s="31" t="inlineStr">
+      <c r="I14" s="31" t="n"/>
+      <c r="J14" s="31" t="inlineStr">
         <is>
           <t>Roll out PAM with just-in-time access; complete least-privilege access recertification</t>
         </is>
       </c>
-      <c r="J14" s="31" t="inlineStr">
+      <c r="K14" s="31" t="inlineStr">
         <is>
           <t>IAM Manager</t>
         </is>
@@ -1190,12 +1199,13 @@
         <f>IF(G15="","",IF(G15&gt;=2,"High",IF(G15=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I15" s="31" t="inlineStr">
+      <c r="I15" s="31" t="n"/>
+      <c r="J15" s="31" t="inlineStr">
         <is>
           <t>Move to quarterly training cadence with role-based modules for high-risk groups</t>
         </is>
       </c>
-      <c r="J15" s="31" t="inlineStr">
+      <c r="K15" s="31" t="inlineStr">
         <is>
           <t>Security Awareness Lead</t>
         </is>
@@ -1236,12 +1246,13 @@
         <f>IF(G16="","",IF(G16&gt;=2,"High",IF(G16=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I16" s="31" t="inlineStr">
+      <c r="I16" s="31" t="n"/>
+      <c r="J16" s="31" t="inlineStr">
         <is>
           <t>Complete encryption-at-rest remediation for all PHI-containing systems; enforce via policy and automated scanning</t>
         </is>
       </c>
-      <c r="J16" s="31" t="inlineStr">
+      <c r="K16" s="31" t="inlineStr">
         <is>
           <t>Data Governance Lead</t>
         </is>
@@ -1282,12 +1293,13 @@
         <f>IF(G17="","",IF(G17&gt;=2,"High",IF(G17=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I17" s="31" t="inlineStr">
+      <c r="I17" s="31" t="n"/>
+      <c r="J17" s="31" t="inlineStr">
         <is>
           <t>Deploy continuous cloud security posture management (CSPM) with automated guardrails</t>
         </is>
       </c>
-      <c r="J17" s="31" t="inlineStr">
+      <c r="K17" s="31" t="inlineStr">
         <is>
           <t>Cloud Security Engineer</t>
         </is>
@@ -1328,12 +1340,13 @@
         <f>IF(G18="","",IF(G18&gt;=2,"High",IF(G18=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I18" s="31" t="inlineStr">
+      <c r="I18" s="31" t="n"/>
+      <c r="J18" s="31" t="inlineStr">
         <is>
           <t>Stand up tested multi-region failover; conduct semi-annual DR tabletop exercises</t>
         </is>
       </c>
-      <c r="J18" s="31" t="inlineStr">
+      <c r="K18" s="31" t="inlineStr">
         <is>
           <t>Director of Infrastructure</t>
         </is>
@@ -1374,12 +1387,13 @@
         <f>IF(G19="","",IF(G19&gt;=2,"High",IF(G19=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I19" s="31" t="inlineStr">
+      <c r="I19" s="31" t="n"/>
+      <c r="J19" s="31" t="inlineStr">
         <is>
           <t>Onboard colocation facility logs to SIEM; tune detection rules against MITRE ATT&amp;CK healthcare threat profile</t>
         </is>
       </c>
-      <c r="J19" s="31" t="inlineStr">
+      <c r="K19" s="31" t="inlineStr">
         <is>
           <t>Security Operations Lead</t>
         </is>
@@ -1420,12 +1434,13 @@
         <f>IF(G20="","",IF(G20&gt;=2,"High",IF(G20=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I20" s="31" t="inlineStr">
+      <c r="I20" s="31" t="n"/>
+      <c r="J20" s="31" t="inlineStr">
         <is>
           <t>Maintain current state; revisit staffing model at next headcount planning cycle</t>
         </is>
       </c>
-      <c r="J20" s="31" t="inlineStr">
+      <c r="K20" s="31" t="inlineStr">
         <is>
           <t>Security Operations Lead</t>
         </is>
@@ -1466,12 +1481,13 @@
         <f>IF(G21="","",IF(G21&gt;=2,"High",IF(G21=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I21" s="31" t="inlineStr">
+      <c r="I21" s="31" t="n"/>
+      <c r="J21" s="31" t="inlineStr">
         <is>
           <t>Schedule and conduct IR tabletop exercise; update plan based on findings</t>
         </is>
       </c>
-      <c r="J21" s="31" t="inlineStr">
+      <c r="K21" s="31" t="inlineStr">
         <is>
           <t>Incident Response Lead</t>
         </is>
@@ -1512,12 +1528,13 @@
         <f>IF(G22="","",IF(G22&gt;=2,"High",IF(G22=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I22" s="31" t="inlineStr">
+      <c r="I22" s="31" t="n"/>
+      <c r="J22" s="31" t="inlineStr">
         <is>
           <t>Run breach-notification tabletop scenario involving Legal, Compliance, and Communications</t>
         </is>
       </c>
-      <c r="J22" s="31" t="inlineStr">
+      <c r="K22" s="31" t="inlineStr">
         <is>
           <t>Compliance Officer</t>
         </is>
@@ -1558,12 +1575,13 @@
         <f>IF(G23="","",IF(G23&gt;=2,"High",IF(G23=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I23" s="31" t="inlineStr">
+      <c r="I23" s="31" t="n"/>
+      <c r="J23" s="31" t="inlineStr">
         <is>
           <t>Conduct full-stack recovery exercise measuring actual RTO/RPO against BIA targets</t>
         </is>
       </c>
-      <c r="J23" s="31" t="inlineStr">
+      <c r="K23" s="31" t="inlineStr">
         <is>
           <t>Director of Infrastructure</t>
         </is>
@@ -1604,12 +1622,13 @@
         <f>IF(G24="","",IF(G24&gt;=2,"High",IF(G24=1,"Medium","Low")))</f>
         <v/>
       </c>
-      <c r="I24" s="31" t="inlineStr">
+      <c r="I24" s="31" t="n"/>
+      <c r="J24" s="31" t="inlineStr">
         <is>
           <t>Maintain current state</t>
         </is>
       </c>
-      <c r="J24" s="31" t="inlineStr">
+      <c r="K24" s="31" t="inlineStr">
         <is>
           <t>Communications Lead</t>
         </is>

</xml_diff>